<commit_message>
Added new test case in generator information
</commit_message>
<xml_diff>
--- a/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
+++ b/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c3d21e494d8a5e9/Desktop/octopussas/Excel sheets/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:801_{49D89DEB-75B0-4750-A1CB-25B4F211ACB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8F7FF73-C693-4263-AFF5-A01070D62382}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{C18DE4E6-E2E9-46E6-B631-2790521AEDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Signup365" sheetId="1" r:id="rId1"/>
@@ -25,6 +20,7 @@
     <sheet name="GeneratorInformation" sheetId="7" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="639" uniqueCount="449">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="471">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1392,6 +1388,72 @@
   </si>
   <si>
     <t>Generator Note with specialcharacters</t>
+  </si>
+  <si>
+    <t>TC_58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generator main phone with Input </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generator main phone with alphabets </t>
+  </si>
+  <si>
+    <t>Generator main phone with numbers</t>
+  </si>
+  <si>
+    <t>Generator main phone with specialcharacters</t>
+  </si>
+  <si>
+    <t>Generator main phone with more than 10 digits</t>
+  </si>
+  <si>
+    <t>Generator main phone with short input</t>
+  </si>
+  <si>
+    <t>98766752349040</t>
+  </si>
+  <si>
+    <t>98763</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ext with alphabets </t>
+  </si>
+  <si>
+    <t>7890523</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ext with more than 5 digits </t>
+  </si>
+  <si>
+    <t>Ext with short input</t>
+  </si>
+  <si>
+    <t>7890532</t>
+  </si>
+  <si>
+    <t>TC_72</t>
+  </si>
+  <si>
+    <t>Generator Email with alphabets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generator Email with numbers </t>
+  </si>
+  <si>
+    <t>Generator Email with specialcharacters</t>
+  </si>
+  <si>
+    <t>Generator Email with invalid format</t>
+  </si>
+  <si>
+    <t>Generator Email with valid format</t>
+  </si>
+  <si>
+    <t>test3234@dfs,com</t>
+  </si>
+  <si>
+    <t>test4657@test.com</t>
   </si>
 </sst>
 </file>
@@ -1471,10 +1533,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1806,15 +1864,18 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B6D8AE-3776-4B30-9CCC-A0DDA74A5F86}">
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="36" customWidth="1"/>
     <col min="3" max="3" width="34.21875" customWidth="1"/>
     <col min="4" max="4" width="40.21875" customWidth="1"/>
+    <col min="5" max="5" width="38.6640625" customWidth="1"/>
+    <col min="6" max="6" width="40.5546875" customWidth="1"/>
+    <col min="7" max="7" width="33.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
@@ -1822,7 +1883,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1830,7 +1891,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>15</v>
       </c>
@@ -1841,7 +1902,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>434</v>
       </c>
@@ -1852,7 +1913,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>15</v>
       </c>
@@ -1866,7 +1927,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>437</v>
       </c>
@@ -1880,7 +1941,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>15</v>
       </c>
@@ -1894,7 +1955,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>441</v>
       </c>
@@ -1908,7 +1969,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>15</v>
       </c>
@@ -1922,7 +1983,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>445</v>
       </c>
@@ -1936,7 +1997,143 @@
         <v>238</v>
       </c>
     </row>
+    <row r="16" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>451</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>453</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>449</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C17" t="s">
+        <v>320</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="E17" t="s">
+        <v>238</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>458</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>273</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="C20" t="s">
+        <v>320</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="E20" t="s">
+        <v>238</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>464</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>465</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>466</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>467</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>463</v>
+      </c>
+      <c r="B23" t="s">
+        <v>320</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D23" t="s">
+        <v>238</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>470</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E23" r:id="rId1" xr:uid="{C64EA2FD-60AA-4CAB-AB14-7FEDE422E234}"/>
+    <hyperlink ref="F23" r:id="rId2" xr:uid="{195689F3-AFDB-4B43-B0FD-BEE3438B1F43}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3467,7 +3664,7 @@
         <v>291</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C32" t="s">
         <v>242</v>
@@ -3479,7 +3676,7 @@
         <v>238</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>263</v>
+        <v>459</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>264</v>

</xml_diff>

<commit_message>
updated test cases of generator Information
</commit_message>
<xml_diff>
--- a/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
+++ b/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
@@ -3,7 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{C18DE4E6-E2E9-46E6-B631-2790521AEDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c3d21e494d8a5e9/Desktop/octopussas/Excel sheets/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:801_{C18DE4E6-E2E9-46E6-B631-2790521AEDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2313918-760D-4D2D-AC58-2826DC31A2AF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +25,6 @@
     <sheet name="GeneratorInformation" sheetId="7" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="479">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1454,6 +1458,30 @@
   </si>
   <si>
     <t>test4657@test.com</t>
+  </si>
+  <si>
+    <t>TC_104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Attention with alphabets </t>
+  </si>
+  <si>
+    <t>Attention with numbers</t>
+  </si>
+  <si>
+    <t>Attention with specialcharacters</t>
+  </si>
+  <si>
+    <t>TC_107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Street with alphabets </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Street with numbers </t>
+  </si>
+  <si>
+    <t>TC_114</t>
   </si>
 </sst>
 </file>
@@ -1864,7 +1892,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B6D8AE-3776-4B30-9CCC-A0DDA74A5F86}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -2127,6 +2155,90 @@
       </c>
       <c r="F23" s="2" t="s">
         <v>470</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>473</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>471</v>
+      </c>
+      <c r="B26" t="s">
+        <v>320</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D26" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>476</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>475</v>
+      </c>
+      <c r="B29" t="s">
+        <v>320</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D29" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>478</v>
+      </c>
+      <c r="B32" t="s">
+        <v>320</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D32" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
written test cases till TC_128
</commit_message>
<xml_diff>
--- a/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
+++ b/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c3d21e494d8a5e9/Desktop/octopussas/Excel sheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:801_{C18DE4E6-E2E9-46E6-B631-2790521AEDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2313918-760D-4D2D-AC58-2826DC31A2AF}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:801_{0D684389-1486-4043-9377-E08D38ED56A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFBA2D2C-B6E9-4675-89F0-CFA124473F02}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="479">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="494">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1482,6 +1482,51 @@
   </si>
   <si>
     <t>TC_114</t>
+  </si>
+  <si>
+    <t>TC_119</t>
+  </si>
+  <si>
+    <t>TC_128</t>
+  </si>
+  <si>
+    <t>Zipcode specialcharacters</t>
+  </si>
+  <si>
+    <t>TC_133</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email with alphabets </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email with numbers </t>
+  </si>
+  <si>
+    <t>Email with Invalid format</t>
+  </si>
+  <si>
+    <t>Testing237487,com</t>
+  </si>
+  <si>
+    <t>TC_138</t>
+  </si>
+  <si>
+    <t>9876</t>
+  </si>
+  <si>
+    <t>9876675234376732</t>
+  </si>
+  <si>
+    <t>Phone with short input</t>
+  </si>
+  <si>
+    <t>34877</t>
+  </si>
+  <si>
+    <t>34877476</t>
+  </si>
+  <si>
+    <t>34</t>
   </si>
 </sst>
 </file>
@@ -1892,7 +1937,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B6D8AE-3776-4B30-9CCC-A0DDA74A5F86}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="36" customWidth="1"/>
@@ -2239,6 +2284,176 @@
       </c>
       <c r="D32" t="s">
         <v>238</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>479</v>
+      </c>
+      <c r="B35" t="s">
+        <v>320</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D35" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>480</v>
+      </c>
+      <c r="B38" t="s">
+        <v>320</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D38" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>482</v>
+      </c>
+      <c r="B41" t="s">
+        <v>320</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D41" t="s">
+        <v>238</v>
+      </c>
+      <c r="E41" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E43" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>487</v>
+      </c>
+      <c r="B44" t="s">
+        <v>320</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="D44" t="s">
+        <v>238</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>118</v>
+      </c>
+      <c r="B47" t="s">
+        <v>320</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="D47" t="s">
+        <v>238</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>493</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modified MyProfile, Transporterfile, Servicevehicle
</commit_message>
<xml_diff>
--- a/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
+++ b/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
@@ -3,12 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7c3d21e494d8a5e9/Desktop/octopussas/Excel sheets/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="13_ncr:801_{0D684389-1486-4043-9377-E08D38ED56A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFBA2D2C-B6E9-4675-89F0-CFA124473F02}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{FEFBC803-64AB-40E0-B94E-D794ECAFE0B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,6 +20,7 @@
     <sheet name="GeneratorInformation" sheetId="7" r:id="rId10"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="753" uniqueCount="494">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="496">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1505,9 +1501,6 @@
     <t>Email with Invalid format</t>
   </si>
   <si>
-    <t>Testing237487,com</t>
-  </si>
-  <si>
     <t>TC_138</t>
   </si>
   <si>
@@ -1527,6 +1520,15 @@
   </si>
   <si>
     <t>34</t>
+  </si>
+  <si>
+    <t>Email with Valid format</t>
+  </si>
+  <si>
+    <t>test4909@test.com</t>
+  </si>
+  <si>
+    <t>test@@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -2358,6 +2360,9 @@
       <c r="E40" s="3" t="s">
         <v>485</v>
       </c>
+      <c r="F40" s="3" t="s">
+        <v>493</v>
+      </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
@@ -2373,7 +2378,10 @@
         <v>238</v>
       </c>
       <c r="E41" t="s">
-        <v>486</v>
+        <v>495</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>494</v>
       </c>
     </row>
     <row r="43" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -2393,12 +2401,12 @@
         <v>253</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B44" t="s">
         <v>320</v>
@@ -2410,10 +2418,10 @@
         <v>238</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="46" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -2444,22 +2452,23 @@
         <v>320</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="D47" t="s">
         <v>238</v>
       </c>
       <c r="E47" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="F47" s="1" t="s">
         <v>492</v>
-      </c>
-      <c r="F47" s="1" t="s">
-        <v>493</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E23" r:id="rId1" xr:uid="{C64EA2FD-60AA-4CAB-AB14-7FEDE422E234}"/>
     <hyperlink ref="F23" r:id="rId2" xr:uid="{195689F3-AFDB-4B43-B0FD-BEE3438B1F43}"/>
+    <hyperlink ref="F41" r:id="rId3" xr:uid="{3A1B7B69-EA8B-4107-9B10-83B1BC89E437}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Modified MyProfile, Service Vehicle, Drivers
</commit_message>
<xml_diff>
--- a/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
+++ b/OctopusSaaS_Dev_Nagaveni/Test data/read.xlsx
@@ -1,26 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{FEFBC803-64AB-40E0-B94E-D794ECAFE0B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{F2D2FD1F-9E2E-47CD-B018-3D8613FCE4D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Signup365" sheetId="1" r:id="rId1"/>
     <sheet name="Generator" sheetId="10" r:id="rId2"/>
     <sheet name="Routeassignment" sheetId="3" r:id="rId3"/>
-    <sheet name="TransporterProfile" sheetId="2" r:id="rId4"/>
-    <sheet name="MyProfile" sheetId="4" r:id="rId5"/>
-    <sheet name="Drivers" sheetId="5" r:id="rId6"/>
-    <sheet name="Servicevehicle" sheetId="6" r:id="rId7"/>
-    <sheet name="SatelliteLocation" sheetId="8" r:id="rId8"/>
-    <sheet name="LiveView" sheetId="9" r:id="rId9"/>
-    <sheet name="GeneratorInformation" sheetId="7" r:id="rId10"/>
+    <sheet name="Disposal Facillity" sheetId="11" r:id="rId4"/>
+    <sheet name="Unapplied checks" sheetId="12" r:id="rId5"/>
+    <sheet name="TransporterProfile" sheetId="2" r:id="rId6"/>
+    <sheet name="MyProfile" sheetId="4" r:id="rId7"/>
+    <sheet name="Drivers" sheetId="5" r:id="rId8"/>
+    <sheet name="Servicevehicle" sheetId="6" r:id="rId9"/>
+    <sheet name="SatelliteLocation" sheetId="8" r:id="rId10"/>
+    <sheet name="LiveView" sheetId="9" r:id="rId11"/>
+    <sheet name="GeneratorInformation" sheetId="7" r:id="rId12"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1"/>
+  <oleSize ref="A22:E30"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -30,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="805">
   <si>
     <t>Tc_ID</t>
   </si>
@@ -1267,9 +1269,6 @@
     <t>SDFFg</t>
   </si>
   <si>
-    <t>"2662</t>
-  </si>
-  <si>
     <t>^*()*%#</t>
   </si>
   <si>
@@ -1345,72 +1344,791 @@
     <t>Service is Good</t>
   </si>
   <si>
+    <t>2662</t>
+  </si>
+  <si>
+    <t>TC_028</t>
+  </si>
+  <si>
+    <t>Updated comapany name</t>
+  </si>
+  <si>
+    <t>Comapany 
+display name</t>
+  </si>
+  <si>
+    <t>Comapany display name with valid input</t>
+  </si>
+  <si>
+    <t>Special charcaters</t>
+  </si>
+  <si>
+    <t>TC_29to32</t>
+  </si>
+  <si>
+    <t>Roadster</t>
+  </si>
+  <si>
+    <t>fdfwf</t>
+  </si>
+  <si>
+    <t>152151</t>
+  </si>
+  <si>
+    <t>#$%^&amp;</t>
+  </si>
+  <si>
+    <t>TC_34 to 37</t>
+  </si>
+  <si>
+    <t>General phone number</t>
+  </si>
+  <si>
+    <t>Valid input</t>
+  </si>
+  <si>
+    <t>5258947689</t>
+  </si>
+  <si>
+    <t>jhghj</t>
+  </si>
+  <si>
+    <t>5234589625</t>
+  </si>
+  <si>
+    <t>General phonenumber ext field</t>
+  </si>
+  <si>
+    <t>Valid  input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">More than 5 digits </t>
+  </si>
+  <si>
+    <t>Short input</t>
+  </si>
+  <si>
+    <t>TC_39 to 44</t>
+  </si>
+  <si>
+    <t>23456</t>
+  </si>
+  <si>
+    <t>dfdw</t>
+  </si>
+  <si>
+    <t>26562</t>
+  </si>
+  <si>
+    <t>$%^&amp;</t>
+  </si>
+  <si>
+    <t>58966522</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>Email name</t>
+  </si>
+  <si>
+    <t>ballu</t>
+  </si>
+  <si>
+    <t>Website text field</t>
+  </si>
+  <si>
+    <t>Special acharcaters</t>
+  </si>
+  <si>
+    <t>furwfhi</t>
+  </si>
+  <si>
+    <t>56556</t>
+  </si>
+  <si>
+    <t>%^&amp;*</t>
+  </si>
+  <si>
+    <t>TC_49to51</t>
+  </si>
+  <si>
+    <t>Copy paste input</t>
+  </si>
+  <si>
+    <t>TC_53</t>
+  </si>
+  <si>
+    <t>Start fsical date</t>
+  </si>
+  <si>
+    <t>Business hour Text field</t>
+  </si>
+  <si>
+    <t>Start Facial date text field</t>
+  </si>
+  <si>
+    <t>TC_57to60</t>
+  </si>
+  <si>
+    <t>Input</t>
+  </si>
+  <si>
+    <t>Hi</t>
+  </si>
+  <si>
+    <t>SDghh</t>
+  </si>
+  <si>
+    <t>13454</t>
+  </si>
+  <si>
+    <t>Combination</t>
+  </si>
+  <si>
+    <t>Ab12$%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Doogle Review linnk
+</t>
+  </si>
+  <si>
+    <t>Special char</t>
+  </si>
+  <si>
+    <t>TC_062 to 65</t>
+  </si>
+  <si>
+    <t>DFGHJT</t>
+  </si>
+  <si>
+    <t>7895452</t>
+  </si>
+  <si>
+    <t>%^&amp;*(</t>
+  </si>
+  <si>
+    <t>Invalid input</t>
+  </si>
+  <si>
+    <t>Gh@ygy.com#</t>
+  </si>
+  <si>
+    <t>Valid Format</t>
+  </si>
+  <si>
+    <t>www.amazom.com</t>
+  </si>
+  <si>
+    <t>Satellite loaction Name</t>
+  </si>
+  <si>
+    <t>Satellite location Status Dropdown</t>
+  </si>
+  <si>
+    <t>TC_075</t>
+  </si>
+  <si>
+    <t>hfrbui</t>
+  </si>
+  <si>
+    <t>RegistrationNumber 1 Text field</t>
+  </si>
+  <si>
+    <t>TC_78to 80</t>
+  </si>
+  <si>
+    <t>SDFGH</t>
+  </si>
+  <si>
+    <t>34567</t>
+  </si>
+  <si>
+    <t>$^&amp;*</t>
+  </si>
+  <si>
+    <t>Tc_82 to 84</t>
+  </si>
+  <si>
+    <t>ftybu</t>
+  </si>
+  <si>
+    <t>8561</t>
+  </si>
+  <si>
+    <t>$%^*</t>
+  </si>
+  <si>
+    <t>EPA ID number text field</t>
+  </si>
+  <si>
+    <t>RTGHyhhh</t>
+  </si>
+  <si>
+    <t>852684</t>
+  </si>
+  <si>
+    <t>#$%^</t>
+  </si>
+  <si>
+    <t>TC_86to 88</t>
+  </si>
+  <si>
+    <t>Dot number field</t>
+  </si>
+  <si>
+    <t>tc_89TO91</t>
+  </si>
+  <si>
+    <t>JHGFV</t>
+  </si>
+  <si>
+    <t>865</t>
+  </si>
+  <si>
+    <t>EIN number</t>
+  </si>
+  <si>
+    <t>TC_92to94</t>
+  </si>
+  <si>
+    <t>GFhjjk</t>
+  </si>
+  <si>
+    <t>$%^&amp;*</t>
+  </si>
+  <si>
+    <t>Entity Id number</t>
+  </si>
+  <si>
+    <t>TC_095to97</t>
+  </si>
+  <si>
+    <t>Hjbj</t>
+  </si>
+  <si>
+    <t>45678</t>
+  </si>
+  <si>
+    <t>856369</t>
+  </si>
+  <si>
+    <t>SoS Numbers</t>
+  </si>
+  <si>
+    <t>TC_98to100</t>
+  </si>
+  <si>
+    <t>tfvV</t>
+  </si>
+  <si>
+    <t>3456</t>
+  </si>
+  <si>
+    <t>SIC code</t>
+  </si>
+  <si>
+    <t>TGfghj</t>
+  </si>
+  <si>
+    <t>5896</t>
+  </si>
+  <si>
+    <t>NAICS code</t>
+  </si>
+  <si>
+    <t>guib</t>
+  </si>
+  <si>
+    <t>7556</t>
+  </si>
+  <si>
+    <t>#$%^&amp;*</t>
+  </si>
+  <si>
+    <t>CAGE code</t>
+  </si>
+  <si>
+    <t>TC_101to103</t>
+  </si>
+  <si>
+    <t>TC_104to106</t>
+  </si>
+  <si>
+    <t>T107to 109</t>
+  </si>
+  <si>
+    <t>YGJ</t>
+  </si>
+  <si>
+    <t>$%^</t>
+  </si>
+  <si>
+    <t>Name text field</t>
+  </si>
+  <si>
+    <t>TC_110to112</t>
+  </si>
+  <si>
+    <t>Raj</t>
+  </si>
+  <si>
+    <t>84658</t>
+  </si>
+  <si>
+    <t>TC_114to116</t>
+  </si>
+  <si>
+    <t>KJN</t>
+  </si>
+  <si>
+    <t>3356</t>
+  </si>
+  <si>
+    <t>(*&amp;%^</t>
+  </si>
+  <si>
+    <t>Street text field</t>
+  </si>
+  <si>
+    <t>Valid Street Address</t>
+  </si>
+  <si>
+    <t>1237 3rd Street</t>
+  </si>
+  <si>
+    <t>Suite Text field</t>
+  </si>
+  <si>
+    <t>TC_120to122</t>
+  </si>
+  <si>
+    <t>huenf</t>
+  </si>
+  <si>
+    <t>56464</t>
+  </si>
+  <si>
+    <t>%*($%^**</t>
+  </si>
+  <si>
+    <t>City text field</t>
+  </si>
+  <si>
+    <t>Special Char</t>
+  </si>
+  <si>
+    <t>TC_124to126</t>
+  </si>
+  <si>
+    <t>lnege</t>
+  </si>
+  <si>
+    <t>987</t>
+  </si>
+  <si>
+    <t>^%$#</t>
+  </si>
+  <si>
+    <t>State Txet field</t>
+  </si>
+  <si>
+    <t>TC_129 to 131</t>
+  </si>
+  <si>
+    <t>Fcjbk</t>
+  </si>
+  <si>
+    <t>84889</t>
+  </si>
+  <si>
+    <t>Zip code text field</t>
+  </si>
+  <si>
+    <t>TC_133 to135</t>
+  </si>
+  <si>
+    <t>Iuhnjn</t>
+  </si>
+  <si>
+    <t>2616</t>
+  </si>
+  <si>
+    <t>Email Text field</t>
+  </si>
+  <si>
+    <t>TC_137to140</t>
+  </si>
+  <si>
+    <t>balli123@gmail.com</t>
+  </si>
+  <si>
+    <t>HUIhfur</t>
+  </si>
+  <si>
+    <t>43143</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid </t>
+  </si>
+  <si>
+    <t>com.@@.com</t>
+  </si>
+  <si>
+    <t>Valid mail ID</t>
+  </si>
+  <si>
+    <t>ballu123@gmail.com</t>
+  </si>
+  <si>
+    <t>Phone number Text field</t>
+  </si>
+  <si>
+    <t>TC_144 to 147</t>
+  </si>
+  <si>
+    <t>243643</t>
+  </si>
+  <si>
+    <t>hbhjbef</t>
+  </si>
+  <si>
+    <t>5646548488</t>
+  </si>
+  <si>
+    <t>$%^&amp;*(</t>
+  </si>
+  <si>
+    <t>Ext text field</t>
+  </si>
+  <si>
+    <t>Tc_149 to 152</t>
+  </si>
+  <si>
+    <t>58975</t>
+  </si>
+  <si>
+    <t>ugi</t>
+  </si>
+  <si>
+    <t>85988</t>
+  </si>
+  <si>
+    <t>&amp;^%@</t>
+  </si>
+  <si>
+    <t>More than 5 digits</t>
+  </si>
+  <si>
+    <t>134525</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>Satellite Billing Information</t>
+  </si>
+  <si>
+    <t>Tc_155to 157</t>
+  </si>
+  <si>
+    <t>veggg</t>
+  </si>
+  <si>
+    <t>64864</t>
+  </si>
+  <si>
+    <t>(*^*%</t>
+  </si>
+  <si>
+    <t>Tc_159to161</t>
+  </si>
+  <si>
+    <t>urig</t>
+  </si>
+  <si>
+    <t>564894</t>
+  </si>
+  <si>
+    <t>*&amp;%#@*</t>
+  </si>
+  <si>
+    <t>TC_165 to167</t>
+  </si>
+  <si>
+    <t>bufrei</t>
+  </si>
+  <si>
+    <t>56156</t>
+  </si>
+  <si>
+    <t>%*%$%</t>
+  </si>
+  <si>
+    <t>TC169to171</t>
+  </si>
+  <si>
+    <t>cdgi</t>
+  </si>
+  <si>
+    <t>64861</t>
+  </si>
+  <si>
+    <t>%*^%^$</t>
+  </si>
+  <si>
+    <t>jhcwvdjc</t>
+  </si>
+  <si>
+    <t>684863</t>
+  </si>
+  <si>
+    <t>(&amp;(*&amp;^%</t>
+  </si>
+  <si>
+    <t>Tc_173 to 175</t>
+  </si>
+  <si>
+    <t>TC_177 to 179</t>
+  </si>
+  <si>
+    <t>kjhrwiug</t>
+  </si>
+  <si>
+    <t>86969</t>
+  </si>
+  <si>
+    <t>#$%^*(</t>
+  </si>
+  <si>
+    <t>Valid Input</t>
+  </si>
+  <si>
+    <t>TC_181 to 184</t>
+  </si>
+  <si>
+    <t>charlie123@gmail.com</t>
+  </si>
+  <si>
+    <t>GYJgj</t>
+  </si>
+  <si>
+    <t>547831</t>
+  </si>
+  <si>
+    <t>&amp;*%8758</t>
+  </si>
+  <si>
+    <t>TC_188 to 191</t>
+  </si>
+  <si>
+    <t>5897458962</t>
+  </si>
+  <si>
+    <t>jjkwbv</t>
+  </si>
+  <si>
+    <t>1234568759</t>
+  </si>
+  <si>
+    <t>*%8758</t>
+  </si>
+  <si>
+    <t>invalid format</t>
+  </si>
+  <si>
+    <t>Tc_194 to 199</t>
+  </si>
+  <si>
+    <t>58945</t>
+  </si>
+  <si>
+    <t>fedsvs</t>
+  </si>
+  <si>
+    <t>68454</t>
+  </si>
+  <si>
+    <t>^$&amp;*&amp;</t>
+  </si>
+  <si>
+    <t>589745</t>
+  </si>
+  <si>
+    <t>Valid name</t>
+  </si>
+  <si>
+    <t>Naren</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>90210</t>
+  </si>
+  <si>
+    <t>Exact Phone Number</t>
+  </si>
+  <si>
+    <t>8596478598</t>
+  </si>
+  <si>
+    <t>Dispatch Department</t>
+  </si>
+  <si>
+    <t>invalid input</t>
+  </si>
+  <si>
+    <t>TC_211 to215</t>
+  </si>
+  <si>
+    <t>jcwdc</t>
+  </si>
+  <si>
+    <t>657897</t>
+  </si>
+  <si>
+    <t>&amp;%&amp;$%#</t>
+  </si>
+  <si>
+    <t>.com@.com</t>
+  </si>
+  <si>
+    <t>TC_217to220</t>
+  </si>
+  <si>
+    <t>9305948592</t>
+  </si>
+  <si>
+    <t>wufifrwf</t>
+  </si>
+  <si>
+    <t>23434242433</t>
+  </si>
+  <si>
+    <t>*(&amp;(^*&amp;%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Special char </t>
+  </si>
+  <si>
+    <t>jhqvfew</t>
+  </si>
+  <si>
+    <t>58963</t>
+  </si>
+  <si>
+    <t>%&amp;**%$</t>
+  </si>
+  <si>
+    <t>589632</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>TC_222to228</t>
+  </si>
+  <si>
+    <t>Comapany Display Name</t>
+  </si>
+  <si>
+    <t>Registration number 1</t>
+  </si>
+  <si>
+    <t>General information fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portland </t>
+  </si>
+  <si>
+    <t>5897412563</t>
+  </si>
+  <si>
+    <t>698742</t>
+  </si>
+  <si>
+    <t>Tc_228</t>
+  </si>
+  <si>
+    <t>Dispatch email</t>
+  </si>
+  <si>
+    <t>Dispatch phone</t>
+  </si>
+  <si>
+    <t>naren</t>
+  </si>
+  <si>
+    <t>5896321475</t>
+  </si>
+  <si>
+    <t>Generator Name with numbers</t>
+  </si>
+  <si>
+    <t>Generator Name with specialcharacters</t>
+  </si>
+  <si>
     <t>TC_012</t>
   </si>
   <si>
-    <t>Generator Name with numbers</t>
-  </si>
-  <si>
-    <t>Generator Name with specialcharacters</t>
+    <t>Internal account number with alphabets</t>
+  </si>
+  <si>
+    <t>Internal account number with numbers</t>
+  </si>
+  <si>
+    <t>Internal account number with specialcharacters</t>
   </si>
   <si>
     <t>TC_018</t>
   </si>
   <si>
-    <t>Internal account number with alphabets</t>
-  </si>
-  <si>
-    <t>Internal account number with numbers</t>
-  </si>
-  <si>
-    <t>Internal account number with specialcharacters</t>
+    <t>Generator permit number with alphabets</t>
+  </si>
+  <si>
+    <t>Generator permit number with numbers</t>
+  </si>
+  <si>
+    <t>Generator permit number with specialcharacters</t>
   </si>
   <si>
     <t>TC_023</t>
   </si>
   <si>
-    <t>Generator permit number with alphabets</t>
-  </si>
-  <si>
-    <t>Generator permit number with numbers</t>
-  </si>
-  <si>
-    <t>Generator permit number with specialcharacters</t>
+    <t>Generator Note with alphabets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generator Note with numbers </t>
+  </si>
+  <si>
+    <t>Generator Note with specialcharacters</t>
   </si>
   <si>
     <t>TC_040</t>
   </si>
   <si>
-    <t>Generator Note with alphabets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generator Note with numbers </t>
-  </si>
-  <si>
-    <t>Generator Note with specialcharacters</t>
+    <t xml:space="preserve">Generator main phone with Input </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generator main phone with alphabets </t>
+  </si>
+  <si>
+    <t>Generator main phone with numbers</t>
+  </si>
+  <si>
+    <t>Generator main phone with specialcharacters</t>
+  </si>
+  <si>
+    <t>Generator main phone with more than 10 digits</t>
+  </si>
+  <si>
+    <t>Generator main phone with short input</t>
   </si>
   <si>
     <t>TC_58</t>
   </si>
   <si>
-    <t xml:space="preserve">Generator main phone with Input </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generator main phone with alphabets </t>
-  </si>
-  <si>
-    <t>Generator main phone with numbers</t>
-  </si>
-  <si>
-    <t>Generator main phone with specialcharacters</t>
-  </si>
-  <si>
-    <t>Generator main phone with more than 10 digits</t>
-  </si>
-  <si>
-    <t>Generator main phone with short input</t>
-  </si>
-  <si>
     <t>98766752349040</t>
   </si>
   <si>
@@ -1420,9 +2138,6 @@
     <t xml:space="preserve">Ext with alphabets </t>
   </si>
   <si>
-    <t>7890523</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ext with more than 5 digits </t>
   </si>
   <si>
@@ -1432,87 +2147,90 @@
     <t>7890532</t>
   </si>
   <si>
+    <t>Generator Email with alphabets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generator Email with numbers </t>
+  </si>
+  <si>
+    <t>Generator Email with specialcharacters</t>
+  </si>
+  <si>
+    <t>Generator Email with invalid format</t>
+  </si>
+  <si>
+    <t>Generator Email with valid format</t>
+  </si>
+  <si>
     <t>TC_72</t>
   </si>
   <si>
-    <t>Generator Email with alphabets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generator Email with numbers </t>
-  </si>
-  <si>
-    <t>Generator Email with specialcharacters</t>
-  </si>
-  <si>
-    <t>Generator Email with invalid format</t>
-  </si>
-  <si>
-    <t>Generator Email with valid format</t>
-  </si>
-  <si>
     <t>test3234@dfs,com</t>
   </si>
   <si>
     <t>test4657@test.com</t>
   </si>
   <si>
+    <t xml:space="preserve">Attention with alphabets </t>
+  </si>
+  <si>
+    <t>Attention with numbers</t>
+  </si>
+  <si>
+    <t>Attention with specialcharacters</t>
+  </si>
+  <si>
     <t>TC_104</t>
   </si>
   <si>
-    <t xml:space="preserve">Attention with alphabets </t>
-  </si>
-  <si>
-    <t>Attention with numbers</t>
-  </si>
-  <si>
-    <t>Attention with specialcharacters</t>
+    <t xml:space="preserve">Street with alphabets </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Street with numbers </t>
   </si>
   <si>
     <t>TC_107</t>
   </si>
   <si>
-    <t xml:space="preserve">Street with alphabets </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Street with numbers </t>
-  </si>
-  <si>
     <t>TC_114</t>
   </si>
   <si>
     <t>TC_119</t>
   </si>
   <si>
+    <t>Zipcode specialcharacters</t>
+  </si>
+  <si>
     <t>TC_128</t>
   </si>
   <si>
-    <t>Zipcode specialcharacters</t>
+    <t xml:space="preserve">Email with alphabets </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email with numbers </t>
+  </si>
+  <si>
+    <t>Email with Invalid format</t>
   </si>
   <si>
     <t>TC_133</t>
   </si>
   <si>
-    <t xml:space="preserve">Email with alphabets </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email with numbers </t>
-  </si>
-  <si>
-    <t>Email with Invalid format</t>
+    <t>Testing237487,com</t>
+  </si>
+  <si>
+    <t>Phone with short input</t>
   </si>
   <si>
     <t>TC_138</t>
   </si>
   <si>
+    <t>9876675234376732</t>
+  </si>
+  <si>
     <t>9876</t>
   </si>
   <si>
-    <t>9876675234376732</t>
-  </si>
-  <si>
-    <t>Phone with short input</t>
-  </si>
-  <si>
     <t>34877</t>
   </si>
   <si>
@@ -1522,13 +2240,226 @@
     <t>34</t>
   </si>
   <si>
-    <t>Email with Valid format</t>
-  </si>
-  <si>
-    <t>test4909@test.com</t>
-  </si>
-  <si>
-    <t>test@@gmail.com</t>
+    <t>Inputs</t>
+  </si>
+  <si>
+    <t>TC_004 to 007</t>
+  </si>
+  <si>
+    <t>Jaxon Reed</t>
+  </si>
+  <si>
+    <t>vlfj</t>
+  </si>
+  <si>
+    <t>16516</t>
+  </si>
+  <si>
+    <t>#$%^&amp;*(</t>
+  </si>
+  <si>
+    <t>jaxnon123@gmail.com</t>
+  </si>
+  <si>
+    <t>hjwbdvw</t>
+  </si>
+  <si>
+    <t>8943</t>
+  </si>
+  <si>
+    <t>TC_009 to 013</t>
+  </si>
+  <si>
+    <t>Invalid format</t>
+  </si>
+  <si>
+    <t>Notification type DD</t>
+  </si>
+  <si>
+    <t>TC_016</t>
+  </si>
+  <si>
+    <t>fruguy</t>
+  </si>
+  <si>
+    <t>.com@</t>
+  </si>
+  <si>
+    <t>Editable Name</t>
+  </si>
+  <si>
+    <t>TC_027</t>
+  </si>
+  <si>
+    <t>Edit name</t>
+  </si>
+  <si>
+    <t>Street Text field</t>
+  </si>
+  <si>
+    <t>TC_029 to32</t>
+  </si>
+  <si>
+    <t>1234 55th Street Northeast</t>
+  </si>
+  <si>
+    <t>sfdafeq</t>
+  </si>
+  <si>
+    <t>48648486</t>
+  </si>
+  <si>
+    <t>Suggestion</t>
+  </si>
+  <si>
+    <t>1234 5</t>
+  </si>
+  <si>
+    <t>Suite text field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numbers </t>
+  </si>
+  <si>
+    <t>TC_037 to40</t>
+  </si>
+  <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>njfknfjke</t>
+  </si>
+  <si>
+    <t>12345</t>
+  </si>
+  <si>
+    <t xml:space="preserve">City Text field </t>
+  </si>
+  <si>
+    <t>special Char</t>
+  </si>
+  <si>
+    <t>TC_043 to46</t>
+  </si>
+  <si>
+    <t>Conton</t>
+  </si>
+  <si>
+    <t>fbwhj</t>
+  </si>
+  <si>
+    <t>6985669</t>
+  </si>
+  <si>
+    <t>State text field</t>
+  </si>
+  <si>
+    <t>Ball</t>
+  </si>
+  <si>
+    <t>TC_049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zip code text field </t>
+  </si>
+  <si>
+    <t>TC_053 to 56</t>
+  </si>
+  <si>
+    <t>589532</t>
+  </si>
+  <si>
+    <t>jkfhf</t>
+  </si>
+  <si>
+    <t>568495</t>
+  </si>
+  <si>
+    <t>Phone field</t>
+  </si>
+  <si>
+    <t>TC_061 to 64</t>
+  </si>
+  <si>
+    <t>5664896525</t>
+  </si>
+  <si>
+    <t>uhfuwhf</t>
+  </si>
+  <si>
+    <t>2556465456</t>
+  </si>
+  <si>
+    <t>Ext field</t>
+  </si>
+  <si>
+    <t>TC_066 to 69</t>
+  </si>
+  <si>
+    <t>546</t>
+  </si>
+  <si>
+    <t>gwrjoi</t>
+  </si>
+  <si>
+    <t>8742</t>
+  </si>
+  <si>
+    <t>!@#$</t>
+  </si>
+  <si>
+    <t>Short Input</t>
+  </si>
+  <si>
+    <t>8898465</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>Dispoasl Facility Dropdown</t>
+  </si>
+  <si>
+    <t>Tc_074</t>
+  </si>
+  <si>
+    <t>Email1 Text field</t>
+  </si>
+  <si>
+    <t>TC_078 tp 80</t>
+  </si>
+  <si>
+    <t>bvfbibv</t>
+  </si>
+  <si>
+    <t>7896533</t>
+  </si>
+  <si>
+    <t>Green Waste Management</t>
+  </si>
+  <si>
+    <t>Account Number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emial ID </t>
+  </si>
+  <si>
+    <t>greenwaste123@gmail.com</t>
+  </si>
+  <si>
+    <t>Phone Number</t>
+  </si>
+  <si>
+    <t>8965741235</t>
+  </si>
+  <si>
+    <t>Charlie waste Management_106893</t>
+  </si>
+  <si>
+    <t>charlie44636</t>
   </si>
 </sst>
 </file>
@@ -1552,7 +2483,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1562,6 +2493,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1579,7 +2516,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -1588,9 +2525,32 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1938,6 +2898,1549 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
+  <dimension ref="A1:H106"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="30.44140625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="25" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="20.77734375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="23.5546875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" style="6" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>391</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>393</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>433</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="6" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>436</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>439</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>440</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>442</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" s="4" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>444</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>449</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="4" customFormat="1" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>451</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>454</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>455</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>456</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>457</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>459</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B25" s="6" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>463</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>466</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>473</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>478</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" s="4" customFormat="1" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F35" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>489</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>484</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>485</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>488</v>
+      </c>
+      <c r="G36" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>498</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>502</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>504</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>506</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>510</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>512</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>521</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>520</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>525</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A55" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="C55" s="8" t="s">
+        <v>528</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
+        <v>529</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A57" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="C57" s="8" t="s">
+        <v>531</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A59" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="C59" s="8" t="s">
+        <v>498</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A61" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="C61" s="8" t="s">
+        <v>542</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A63" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="C63" s="8" t="s">
+        <v>545</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A65" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="C65" s="8" t="s">
+        <v>553</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A67" s="6" t="s">
+        <v>557</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="C67" s="8" t="s">
+        <v>559</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A69" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="C69" s="8" t="s">
+        <v>564</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="4" t="s">
+        <v>565</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A71" s="6" t="s">
+        <v>566</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>568</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>486</v>
+      </c>
+      <c r="E71" s="8" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>574</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="H72" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A73" s="6" t="s">
+        <v>570</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>571</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>572</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>573</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>575</v>
+      </c>
+      <c r="G73" s="9" t="s">
+        <v>577</v>
+      </c>
+      <c r="H73" s="6" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A75" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>580</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>581</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>582</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>583</v>
+      </c>
+      <c r="F75" s="8" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="G76" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A77" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>586</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>588</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>589</v>
+      </c>
+      <c r="F77" s="8" t="s">
+        <v>591</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A78" s="10" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="4" t="s">
+        <v>539</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A80" s="6" t="s">
+        <v>594</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>596</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A82" s="6" t="s">
+        <v>598</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>600</v>
+      </c>
+      <c r="D82" s="9" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A84" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>604</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A86" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>607</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>608</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" s="6" t="s">
+        <v>613</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>611</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="4" t="s">
+        <v>565</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>616</v>
+      </c>
+      <c r="D90" s="6" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>618</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="G91" s="4" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A92" s="6" t="s">
+        <v>619</v>
+      </c>
+      <c r="B92" s="9" t="s">
+        <v>620</v>
+      </c>
+      <c r="C92" s="6" t="s">
+        <v>621</v>
+      </c>
+      <c r="D92" s="8" t="s">
+        <v>622</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>623</v>
+      </c>
+      <c r="F92" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="G92" s="9" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="B94" s="8" t="s">
+        <v>625</v>
+      </c>
+      <c r="C94" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="D94" s="8" t="s">
+        <v>627</v>
+      </c>
+      <c r="E94" s="6" t="s">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>618</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="B96" s="8" t="s">
+        <v>631</v>
+      </c>
+      <c r="C96" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="D96" s="8" t="s">
+        <v>633</v>
+      </c>
+      <c r="E96" s="6" t="s">
+        <v>634</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>635</v>
+      </c>
+      <c r="G96" s="8" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" s="10" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>482</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>643</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="B99" s="8" t="s">
+        <v>620</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="D99" s="8" t="s">
+        <v>646</v>
+      </c>
+      <c r="E99" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="F99" s="9" t="s">
+        <v>648</v>
+      </c>
+      <c r="G99" s="9" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="B101" s="8" t="s">
+        <v>650</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>651</v>
+      </c>
+      <c r="D101" s="8" t="s">
+        <v>652</v>
+      </c>
+      <c r="E101" s="6" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="E102" s="4" t="s">
+        <v>654</v>
+      </c>
+      <c r="F102" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="G102" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="B103" s="8" t="s">
+        <v>586</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="D103" s="8" t="s">
+        <v>656</v>
+      </c>
+      <c r="E103" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="F103" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="G103" s="8" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" s="4" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A105" s="4" t="s">
+        <v>663</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>661</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>662</v>
+      </c>
+      <c r="E105" s="4" t="s">
+        <v>668</v>
+      </c>
+      <c r="F105" s="4" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A106" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="C106" s="8" t="s">
+        <v>665</v>
+      </c>
+      <c r="D106" s="8" t="s">
+        <v>666</v>
+      </c>
+      <c r="E106" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>671</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" display="#$%@$%" xr:uid="{5A227241-ECE1-4878-A7FE-E1EBF1CFB34A}"/>
+    <hyperlink ref="B6" r:id="rId2" xr:uid="{284322BF-D005-4BF8-9C8A-1D78ADDFD986}"/>
+    <hyperlink ref="E6" r:id="rId3" xr:uid="{77471F4F-AA24-4166-BB1C-7C0B003FB5F7}"/>
+    <hyperlink ref="B10" r:id="rId4" xr:uid="{A5A7610F-A733-45B6-90BA-72F05DA28534}"/>
+    <hyperlink ref="E28" r:id="rId5" xr:uid="{1269199C-B882-4CF4-8FE7-B5632B815114}"/>
+    <hyperlink ref="B36" r:id="rId6" xr:uid="{F80053D1-6192-46D4-8135-3162E9DCDBFF}"/>
+    <hyperlink ref="F36" r:id="rId7" xr:uid="{A2E87AD7-519E-4D64-A8B0-804F45B567E3}"/>
+    <hyperlink ref="G36" r:id="rId8" xr:uid="{001C606C-950A-42AD-84B8-A6A9B9513EE9}"/>
+    <hyperlink ref="B73" r:id="rId9" xr:uid="{24CFF544-36E4-4F50-A277-C01ABB4FEEC2}"/>
+    <hyperlink ref="F73" r:id="rId10" display="com@" xr:uid="{C8CFEF57-B152-49C3-AFFA-70B8D30BAEEE}"/>
+    <hyperlink ref="G73" r:id="rId11" xr:uid="{ACEECA67-88F7-427D-BFAF-783DE7661C96}"/>
+    <hyperlink ref="E77" r:id="rId12" xr:uid="{4E986B8C-EDF0-45DA-B387-2BAFD2E8026F}"/>
+    <hyperlink ref="D82" r:id="rId13" xr:uid="{CDD6978D-1DF9-47A7-99E0-AA10BDC906A5}"/>
+    <hyperlink ref="B92" r:id="rId14" xr:uid="{15FDAB5F-0AF4-4F79-8B5D-CA436D3B9DC1}"/>
+    <hyperlink ref="G92" r:id="rId15" xr:uid="{224A48AA-0076-41B6-B0C3-F943D56C406C}"/>
+    <hyperlink ref="F99" r:id="rId16" xr:uid="{10706437-A8D3-431D-AB38-0D11EC24B8B2}"/>
+    <hyperlink ref="G99" r:id="rId17" display="charlie123@gmail.com" xr:uid="{BE1272E6-3091-460B-92B3-2F7568D11C99}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91B8B5A6-41F7-4B76-9B90-A5C1587D6738}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="11.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>412</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4B6D8AE-3776-4B30-9CCC-A0DDA74A5F86}">
   <dimension ref="A1:G47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1971,15 +4474,15 @@
         <v>15</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>435</v>
+        <v>672</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>436</v>
+        <v>673</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>434</v>
+        <v>674</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>321</v>
@@ -1993,18 +4496,18 @@
         <v>15</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>438</v>
+        <v>675</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>439</v>
+        <v>676</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>440</v>
+        <v>677</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>437</v>
+        <v>678</v>
       </c>
       <c r="B8" t="s">
         <v>320</v>
@@ -2021,18 +4524,18 @@
         <v>15</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>442</v>
+        <v>679</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>443</v>
+        <v>680</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>444</v>
+        <v>681</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>441</v>
+        <v>682</v>
       </c>
       <c r="B11" t="s">
         <v>320</v>
@@ -2049,18 +4552,18 @@
         <v>15</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>446</v>
+        <v>683</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>447</v>
+        <v>684</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>448</v>
+        <v>685</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>445</v>
+        <v>686</v>
       </c>
       <c r="B14" t="s">
         <v>320</v>
@@ -2077,27 +4580,27 @@
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>450</v>
+        <v>687</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>451</v>
+        <v>688</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>452</v>
+        <v>689</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>453</v>
+        <v>690</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>454</v>
+        <v>691</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>455</v>
+        <v>692</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>449</v>
+        <v>693</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>256</v>
@@ -2112,10 +4615,10 @@
         <v>238</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>456</v>
+        <v>694</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>457</v>
+        <v>695</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -2126,7 +4629,7 @@
         <v>228</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>458</v>
+        <v>696</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>158</v>
@@ -2135,10 +4638,10 @@
         <v>159</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>460</v>
+        <v>697</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>461</v>
+        <v>698</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
@@ -2158,7 +4661,7 @@
         <v>238</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>462</v>
+        <v>699</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>264</v>
@@ -2169,24 +4672,24 @@
         <v>15</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>464</v>
+        <v>700</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>465</v>
+        <v>701</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>466</v>
+        <v>702</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>467</v>
+        <v>703</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>468</v>
+        <v>704</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>463</v>
+        <v>705</v>
       </c>
       <c r="B23" t="s">
         <v>320</v>
@@ -2198,10 +4701,10 @@
         <v>238</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>469</v>
+        <v>706</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>470</v>
+        <v>707</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -2209,18 +4712,18 @@
         <v>15</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>472</v>
+        <v>708</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>473</v>
+        <v>709</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>474</v>
+        <v>710</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>471</v>
+        <v>711</v>
       </c>
       <c r="B26" t="s">
         <v>320</v>
@@ -2237,10 +4740,10 @@
         <v>15</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>476</v>
+        <v>712</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>477</v>
+        <v>713</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>99</v>
@@ -2248,7 +4751,7 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>475</v>
+        <v>714</v>
       </c>
       <c r="B29" t="s">
         <v>320</v>
@@ -2276,7 +4779,7 @@
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>478</v>
+        <v>715</v>
       </c>
       <c r="B32" t="s">
         <v>320</v>
@@ -2304,7 +4807,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>479</v>
+        <v>716</v>
       </c>
       <c r="B35" t="s">
         <v>320</v>
@@ -2327,12 +4830,12 @@
         <v>129</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>481</v>
+        <v>717</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>480</v>
+        <v>718</v>
       </c>
       <c r="B38" t="s">
         <v>320</v>
@@ -2349,24 +4852,21 @@
         <v>15</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>483</v>
+        <v>719</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>484</v>
+        <v>720</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>138</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>485</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>493</v>
+        <v>721</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>482</v>
+        <v>722</v>
       </c>
       <c r="B41" t="s">
         <v>320</v>
@@ -2378,10 +4878,7 @@
         <v>238</v>
       </c>
       <c r="E41" t="s">
-        <v>495</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>494</v>
+        <v>723</v>
       </c>
     </row>
     <row r="43" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -2401,12 +4898,12 @@
         <v>253</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>489</v>
+        <v>724</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>486</v>
+        <v>725</v>
       </c>
       <c r="B44" t="s">
         <v>320</v>
@@ -2418,10 +4915,10 @@
         <v>238</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>488</v>
+        <v>726</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>487</v>
+        <v>727</v>
       </c>
     </row>
     <row r="46" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -2441,7 +4938,7 @@
         <v>260</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>461</v>
+        <v>698</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -2452,23 +4949,22 @@
         <v>320</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>490</v>
+        <v>728</v>
       </c>
       <c r="D47" t="s">
         <v>238</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>491</v>
+        <v>729</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>492</v>
+        <v>730</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E23" r:id="rId1" xr:uid="{C64EA2FD-60AA-4CAB-AB14-7FEDE422E234}"/>
-    <hyperlink ref="F23" r:id="rId2" xr:uid="{195689F3-AFDB-4B43-B0FD-BEE3438B1F43}"/>
-    <hyperlink ref="F41" r:id="rId3" xr:uid="{3A1B7B69-EA8B-4107-9B10-83B1BC89E437}"/>
+    <hyperlink ref="E23" r:id="rId1" xr:uid="{4F8EBCF3-1866-4794-8F4F-9060DF8CC2E9}"/>
+    <hyperlink ref="F23" r:id="rId2" xr:uid="{94686A13-7684-4DC8-AB87-C0C9E54E1546}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2476,10 +4972,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77142416-745D-4F9D-B8CB-E786E8AF6BF4}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -2489,21 +4985,26 @@
         <v>77</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B2" t="s">
         <v>415</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D2" t="s">
         <v>416</v>
       </c>
-      <c r="D2" t="s">
-        <v>417</v>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>803</v>
       </c>
     </row>
   </sheetData>
@@ -2562,19 +5063,19 @@
         <v>15</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>418</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="3" t="s">
         <v>419</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>421</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>422</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -2582,23 +5083,23 @@
       <c r="J4" s="3"/>
     </row>
     <row r="5" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="6" t="s">
+        <v>422</v>
+      </c>
+      <c r="B5" t="s">
         <v>423</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>424</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>425</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>426</v>
       </c>
-      <c r="E5" t="s">
-        <v>427</v>
-      </c>
       <c r="F5" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -2606,7 +5107,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -2619,10 +5120,10 @@
     </row>
     <row r="8" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>428</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>429</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
@@ -2630,7 +5131,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -2643,10 +5144,10 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>431</v>
+      </c>
+      <c r="B11" t="s">
         <v>432</v>
-      </c>
-      <c r="B11" t="s">
-        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -2658,6 +5159,468 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB07B270-85DC-4F6D-8AC7-D93CAE493508}">
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.109375" style="11" customWidth="1"/>
+    <col min="2" max="2" width="15.6640625" style="11" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" style="11" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" style="11" customWidth="1"/>
+    <col min="5" max="5" width="16.77734375" style="11" customWidth="1"/>
+    <col min="6" max="6" width="11.44140625" style="11" customWidth="1"/>
+    <col min="7" max="16384" width="8.88671875" style="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
+        <v>539</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>731</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>732</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>733</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>734</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>735</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>569</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>731</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>556</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
+        <v>740</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>737</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>738</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>739</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>583</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="12" t="s">
+        <v>742</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="11" t="s">
+        <v>743</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="12" t="s">
+        <v>746</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
+        <v>749</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>475</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>482</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A14" s="11" t="s">
+        <v>750</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>751</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>752</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>753</v>
+      </c>
+      <c r="E14" s="11" t="s">
+        <v>532</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="12" t="s">
+        <v>756</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>757</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>758</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="11" t="s">
+        <v>759</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>760</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>761</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>762</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="12" t="s">
+        <v>763</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>757</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>758</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="11" t="s">
+        <v>765</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>766</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>767</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>768</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="12" t="s">
+        <v>769</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="11" t="s">
+        <v>771</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="12" t="s">
+        <v>772</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>757</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>758</v>
+      </c>
+      <c r="E21" s="12" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="11" t="s">
+        <v>773</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>774</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>775</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>776</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="12" t="s">
+        <v>777</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>757</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>758</v>
+      </c>
+      <c r="E23" s="12" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="11" t="s">
+        <v>778</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>779</v>
+      </c>
+      <c r="C24" s="11" t="s">
+        <v>780</v>
+      </c>
+      <c r="D24" s="13" t="s">
+        <v>781</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="12" t="s">
+        <v>782</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>757</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>758</v>
+      </c>
+      <c r="E25" s="12" t="s">
+        <v>556</v>
+      </c>
+      <c r="F25" s="12" t="s">
+        <v>590</v>
+      </c>
+      <c r="G25" s="12" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="11" t="s">
+        <v>783</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>784</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>785</v>
+      </c>
+      <c r="D26" s="13" t="s">
+        <v>786</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>787</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>789</v>
+      </c>
+      <c r="G26" s="13" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="12" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="12" t="s">
+        <v>791</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="11" t="s">
+        <v>792</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="12" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="12" t="s">
+        <v>793</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="11" t="s">
+        <v>794</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>795</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>796</v>
+      </c>
+      <c r="D30" s="11" t="s">
+        <v>583</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{97922CCB-F8DD-49B3-B277-333B7101C873}"/>
+    <hyperlink ref="F5" r:id="rId2" xr:uid="{D0E61A3A-F6C2-4149-AEB4-F40D03F71117}"/>
+    <hyperlink ref="E26" r:id="rId3" xr:uid="{08AD4D6E-B198-4A0A-8B71-76D117D9FEC0}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16196D24-437F-4113-984C-E1E07E6FEFBB}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>798</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>799</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>797</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>800</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>802</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{FA134B35-6A03-43B7-BC3C-F6C686D80E46}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A4B5976-09F6-46A1-AF3B-E9A8DFB4EAF3}">
   <dimension ref="A1:G68"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3449,7 +6412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B476B142-4B93-4B5F-AFDD-C5C6F475C99C}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -3601,7 +6564,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58630B64-2EDF-4356-94B8-66DDB845E6F8}">
   <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4000,7 +6963,7 @@
         <v>291</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C32" t="s">
         <v>242</v>
@@ -4012,7 +6975,7 @@
         <v>238</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>459</v>
+        <v>263</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>264</v>
@@ -4109,7 +7072,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77AFD7FA-CE31-4CAB-9D77-EB9A0F5923D7}">
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -4506,157 +7469,4 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA295969-90AC-4E58-86B0-7D3D7C05400C}">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>386</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>387</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>390</v>
-      </c>
-      <c r="B2" t="s">
-        <v>391</v>
-      </c>
-      <c r="C2" t="s">
-        <v>392</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>393</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>396</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>397</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>399</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>400</v>
-      </c>
-      <c r="C6" t="s">
-        <v>401</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>404</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>406</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>388</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>407</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="C10" t="s">
-        <v>409</v>
-      </c>
-      <c r="D10" t="s">
-        <v>410</v>
-      </c>
-      <c r="E10" t="s">
-        <v>411</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" display="#$%@$%" xr:uid="{5A227241-ECE1-4878-A7FE-E1EBF1CFB34A}"/>
-    <hyperlink ref="B6" r:id="rId2" xr:uid="{284322BF-D005-4BF8-9C8A-1D78ADDFD986}"/>
-    <hyperlink ref="E6" r:id="rId3" xr:uid="{77471F4F-AA24-4166-BB1C-7C0B003FB5F7}"/>
-    <hyperlink ref="B10" r:id="rId4" xr:uid="{A5A7610F-A733-45B6-90BA-72F05DA28534}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91B8B5A6-41F7-4B76-9B90-A5C1587D6738}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="11.21875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>413</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>